<commit_message>
benchmarks: regenerate comparison tables + workbook (ascm/ppscm/cwz now live)
Refreshes every comparison.csv and the combined comparisons.xlsx so the three
cases converted to live reference runs -- ascm_kansas and ppscm_paglayan (live
augsynth) and cwz_ttest (live scinference) -- carry their live-reference numbers
and provenance alongside the other 22 cases.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015nRd88pbMUETcrkKY1S6Hr
</commit_message>
<xml_diff>
--- a/benchmarks/reference/comparisons.xlsx
+++ b/benchmarks/reference/comparisons.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:03:54Z</t>
+          <t>2026-06-24T15:00:46Z</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-06-24T14:04:13Z</t>
+          <t>2026-06-24T15:01:05Z</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>R augsynth::multisynth (via Rscript)</t>
+          <t>R augsynth::multisynth (live run, captured)</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-06-24T14:04:16Z</t>
+          <t>2026-06-24T15:01:08Z</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-06-24T14:04:37Z</t>
+          <t>2026-06-24T15:01:29Z</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-06-24T14:04:41Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:11Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:11Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:12Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:12Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -739,11 +739,11 @@
         <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>0.003903</v>
+        <v>0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:12Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Chernozhukov-Wuthrich-Zhu scinference / Table 5(a)</t>
+          <t>R package scinference (sc.cf t-test, live run, captured)</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:22Z</t>
+          <t>2026-06-24T15:02:43Z</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:24Z</t>
+          <t>2026-06-24T15:02:45Z</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:27Z</t>
+          <t>2026-06-24T15:02:48Z</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:28Z</t>
+          <t>2026-06-24T15:02:48Z</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:31Z</t>
+          <t>2026-06-24T15:02:51Z</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:32Z</t>
+          <t>2026-06-24T15:02:52Z</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:32Z</t>
+          <t>2026-06-24T15:02:52Z</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:32Z</t>
+          <t>2026-06-24T15:02:52Z</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -991,11 +991,11 @@
         <v>8</v>
       </c>
       <c r="C20" t="n">
-        <v>0.002239</v>
+        <v>0.009146</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:32Z</t>
+          <t>2026-06-24T15:02:52Z</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>R package augsynth (Kansas vignette)</t>
+          <t>R package augsynth (live run, Kansas study)</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-06-24T14:07:06Z</t>
+          <t>2026-06-24T15:03:18Z</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-06-24T14:07:21Z</t>
+          <t>2026-06-24T15:03:32Z</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-06-24T14:08:02Z</t>
+          <t>2026-06-24T15:04:04Z</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-06-24T14:08:20Z</t>
+          <t>2026-06-24T15:04:19Z</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-06-24T14:08:20Z</t>
+          <t>2026-06-24T15:04:19Z</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-06-24T14:08:20Z</t>
+          <t>2026-06-24T15:04:20Z</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:12Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:12Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
     </row>
@@ -1747,7 +1747,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chernozhukov-Wuthrich-Zhu scinference / Table 5(a)</t>
+          <t>R package scinference (sc.cf t-test, live run, captured)</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pinned published constants (arXiv:1812.10820, Table 5(a))</t>
+          <t>scinference 0.0.0.9000</t>
         </is>
       </c>
     </row>
@@ -1795,10 +1795,10 @@
         <v>-0.273903</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.27</v>
+        <v>-0.273903</v>
       </c>
       <c r="D10" t="n">
-        <v>0.003903</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1811,10 +1811,10 @@
         <v>-0.406425</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.41</v>
+        <v>-0.406425</v>
       </c>
       <c r="D11" t="n">
-        <v>0.003575</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1827,10 +1827,10 @@
         <v>-0.14138</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.14</v>
+        <v>-0.14138</v>
       </c>
       <c r="D12" t="n">
-        <v>0.00138</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:22Z</t>
+          <t>2026-06-24T15:02:43Z</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:24Z</t>
+          <t>2026-06-24T15:02:45Z</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:27Z</t>
+          <t>2026-06-24T15:02:48Z</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:28Z</t>
+          <t>2026-06-24T15:02:48Z</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:31Z</t>
+          <t>2026-06-24T15:02:51Z</t>
         </is>
       </c>
     </row>
@@ -8515,7 +8515,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:32Z</t>
+          <t>2026-06-24T15:02:52Z</t>
         </is>
       </c>
     </row>
@@ -8843,7 +8843,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:32Z</t>
+          <t>2026-06-24T15:02:52Z</t>
         </is>
       </c>
     </row>
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:32Z</t>
+          <t>2026-06-24T15:02:52Z</t>
         </is>
       </c>
     </row>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:03:54Z</t>
+          <t>2026-06-24T15:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9667,7 +9667,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:06:32Z</t>
+          <t>2026-06-24T15:02:52Z</t>
         </is>
       </c>
     </row>
@@ -9715,7 +9715,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R package augsynth (Kansas vignette)</t>
+          <t>R package augsynth (live run, Kansas study)</t>
         </is>
       </c>
     </row>
@@ -9727,7 +9727,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>augsynth 0.2.0 @ 7a90ea4</t>
+          <t>augsynth 0.2.0</t>
         </is>
       </c>
     </row>
@@ -9763,10 +9763,10 @@
         <v>-0.029435</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.029</v>
+        <v>-0.029435</v>
       </c>
       <c r="D10" t="n">
-        <v>0.000435</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -9779,10 +9779,10 @@
         <v>0.082555</v>
       </c>
       <c r="C11" t="n">
-        <v>0.083</v>
+        <v>0.082555</v>
       </c>
       <c r="D11" t="n">
-        <v>0.000445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -9795,10 +9795,10 @@
         <v>-0.040063</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.04</v>
+        <v>-0.040063</v>
       </c>
       <c r="D12" t="n">
-        <v>6.3e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -9811,10 +9811,10 @@
         <v>0.061515</v>
       </c>
       <c r="C13" t="n">
-        <v>0.062</v>
+        <v>0.061515</v>
       </c>
       <c r="D13" t="n">
-        <v>0.000485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -9827,10 +9827,10 @@
         <v>-0.062904</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.061</v>
+        <v>-0.060937</v>
       </c>
       <c r="D14" t="n">
-        <v>0.001904</v>
+        <v>0.001967</v>
       </c>
     </row>
     <row r="15">
@@ -9843,10 +9843,10 @@
         <v>0.054591</v>
       </c>
       <c r="C15" t="n">
-        <v>0.054</v>
+        <v>0.053855</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0005910000000000001</v>
+        <v>0.000736</v>
       </c>
     </row>
     <row r="16">
@@ -9859,10 +9859,10 @@
         <v>-0.057239</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.055</v>
+        <v>-0.052773</v>
       </c>
       <c r="D16" t="n">
-        <v>0.002239</v>
+        <v>0.004466</v>
       </c>
     </row>
     <row r="17">
@@ -9875,10 +9875,10 @@
         <v>0.066783</v>
       </c>
       <c r="C17" t="n">
-        <v>0.067</v>
+        <v>0.057637</v>
       </c>
       <c r="D17" t="n">
-        <v>0.000217</v>
+        <v>0.009146</v>
       </c>
     </row>
   </sheetData>
@@ -9915,7 +9915,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:07:06Z</t>
+          <t>2026-06-24T15:03:18Z</t>
         </is>
       </c>
     </row>
@@ -10275,7 +10275,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:07:21Z</t>
+          <t>2026-06-24T15:03:32Z</t>
         </is>
       </c>
     </row>
@@ -10443,7 +10443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:08:02Z</t>
+          <t>2026-06-24T15:04:04Z</t>
         </is>
       </c>
     </row>
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:08:20Z</t>
+          <t>2026-06-24T15:04:19Z</t>
         </is>
       </c>
     </row>
@@ -11019,7 +11019,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:08:20Z</t>
+          <t>2026-06-24T15:04:19Z</t>
         </is>
       </c>
     </row>
@@ -11379,7 +11379,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:08:20Z</t>
+          <t>2026-06-24T15:04:20Z</t>
         </is>
       </c>
     </row>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:04:13Z</t>
+          <t>2026-06-24T15:01:05Z</t>
         </is>
       </c>
     </row>
@@ -11687,7 +11687,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R augsynth::multisynth (via Rscript)</t>
+          <t>R augsynth::multisynth (live run, captured)</t>
         </is>
       </c>
     </row>
@@ -11699,7 +11699,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>augsynth (R, live)</t>
+          <t>augsynth 0.2.0</t>
         </is>
       </c>
     </row>
@@ -11751,10 +11751,10 @@
         <v>-0.011</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.011</v>
+        <v>-0.0112</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="12">
@@ -11767,10 +11767,10 @@
         <v>0.0026</v>
       </c>
       <c r="C12" t="n">
-        <v>0.003</v>
+        <v>0.0026</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -11799,10 +11799,10 @@
         <v>-0.017</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.018</v>
+        <v>-0.0182</v>
       </c>
       <c r="D14" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
     </row>
     <row r="15">
@@ -11815,10 +11815,10 @@
         <v>-0.004336</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.004282</v>
+        <v>-0.0043</v>
       </c>
       <c r="D15" t="n">
-        <v>5.4e-05</v>
+        <v>3.6e-05</v>
       </c>
     </row>
     <row r="16">
@@ -11831,10 +11831,10 @@
         <v>-0.010699</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.010857</v>
+        <v>-0.010858</v>
       </c>
       <c r="D16" t="n">
-        <v>0.000158</v>
+        <v>0.000159</v>
       </c>
     </row>
     <row r="17">
@@ -11847,10 +11847,10 @@
         <v>0.004367</v>
       </c>
       <c r="C17" t="n">
-        <v>0.004379</v>
+        <v>0.00442</v>
       </c>
       <c r="D17" t="n">
-        <v>1.2e-05</v>
+        <v>5.3e-05</v>
       </c>
     </row>
     <row r="18">
@@ -11863,10 +11863,10 @@
         <v>0.001388</v>
       </c>
       <c r="C18" t="n">
-        <v>0.001155</v>
+        <v>0.001149</v>
       </c>
       <c r="D18" t="n">
-        <v>0.000233</v>
+        <v>0.000239</v>
       </c>
     </row>
     <row r="19">
@@ -11879,10 +11879,10 @@
         <v>-0.009072999999999999</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.009305000000000001</v>
+        <v>-0.009252</v>
       </c>
       <c r="D19" t="n">
-        <v>0.000232</v>
+        <v>0.000179</v>
       </c>
     </row>
     <row r="20">
@@ -11895,10 +11895,10 @@
         <v>-0.016488</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.016943</v>
+        <v>-0.016837</v>
       </c>
       <c r="D20" t="n">
-        <v>0.000455</v>
+        <v>0.000349</v>
       </c>
     </row>
     <row r="21">
@@ -11911,10 +11911,10 @@
         <v>-0.018164</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.018505</v>
+        <v>-0.018476</v>
       </c>
       <c r="D21" t="n">
-        <v>0.000341</v>
+        <v>0.000312</v>
       </c>
     </row>
     <row r="22">
@@ -11927,10 +11927,10 @@
         <v>-0.003424</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.003867</v>
+        <v>-0.003846</v>
       </c>
       <c r="D22" t="n">
-        <v>0.000443</v>
+        <v>0.000422</v>
       </c>
     </row>
     <row r="23">
@@ -11943,10 +11943,10 @@
         <v>-0.015579</v>
       </c>
       <c r="C23" t="n">
-        <v>-0.015836</v>
+        <v>-0.0158</v>
       </c>
       <c r="D23" t="n">
-        <v>0.000257</v>
+        <v>0.000221</v>
       </c>
     </row>
     <row r="24">
@@ -11959,10 +11959,10 @@
         <v>-0.031283</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.031751</v>
+        <v>-0.031627</v>
       </c>
       <c r="D24" t="n">
-        <v>0.000468</v>
+        <v>0.000344</v>
       </c>
     </row>
     <row r="25">
@@ -11975,10 +11975,10 @@
         <v>-0.01734</v>
       </c>
       <c r="C25" t="n">
-        <v>-0.017839</v>
+        <v>-0.017657</v>
       </c>
       <c r="D25" t="n">
-        <v>0.000499</v>
+        <v>0.000317</v>
       </c>
     </row>
     <row r="26">
@@ -12183,10 +12183,10 @@
         <v>0.01565</v>
       </c>
       <c r="C38" t="n">
-        <v>0.01553</v>
+        <v>0.01554</v>
       </c>
       <c r="D38" t="n">
-        <v>0.00012</v>
+        <v>0.00011</v>
       </c>
     </row>
     <row r="39">
@@ -12391,10 +12391,10 @@
         <v>0.02395</v>
       </c>
       <c r="C51" t="n">
-        <v>0.02461</v>
+        <v>0.0246</v>
       </c>
       <c r="D51" t="n">
-        <v>0.00066</v>
+        <v>0.00065</v>
       </c>
     </row>
     <row r="52">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:04:16Z</t>
+          <t>2026-06-24T15:01:08Z</t>
         </is>
       </c>
     </row>
@@ -12679,7 +12679,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:04:37Z</t>
+          <t>2026-06-24T15:01:29Z</t>
         </is>
       </c>
     </row>
@@ -12815,7 +12815,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:04:41Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
     </row>
@@ -13255,7 +13255,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:11Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
     </row>
@@ -13471,7 +13471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:11Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
     </row>
@@ -13751,7 +13751,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T14:05:12Z</t>
+          <t>2026-06-24T15:01:33Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild comparison workbook + CSVs with three live reference conversions
Run the full export so the side-by-side comparison artifacts reflect the
malo_basque, mscmt_basque, and orthsc_carbontax cases now cross-validating
against live captured reference runs (scm.corner, MSCMT, Fry ORTHSC) rather
than hand-pinned constants. comparisons.xlsx now carries 25 case sheets.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/reference/comparisons.xlsx
+++ b/benchmarks/reference/comparisons.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:00:46Z</t>
+          <t>2026-06-24T15:26:35Z</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:05Z</t>
+          <t>2026-06-24T15:26:53Z</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:08Z</t>
+          <t>2026-06-24T15:26:56Z</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:29Z</t>
+          <t>2026-06-24T15:27:18Z</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:22Z</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:22Z</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:22Z</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:22Z</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:23Z</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:23Z</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -767,11 +767,11 @@
         <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>4.1e-05</v>
+        <v>4e-05</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:43Z</t>
+          <t>2026-06-24T15:28:31Z</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>R package MSCMT (vignette)</t>
+          <t>R package MSCMT (live run, captured)</t>
         </is>
       </c>
     </row>
@@ -795,11 +795,11 @@
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>0.000445</v>
+        <v>0.000481</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:45Z</t>
+          <t>2026-06-24T15:28:34Z</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Malo et al. scm.corner (SCM-Debug)</t>
+          <t>Malo et al. scm.corner (SCM-Debug, live run, captured)</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:48Z</t>
+          <t>2026-06-24T15:28:36Z</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:48Z</t>
+          <t>2026-06-24T15:28:37Z</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:51Z</t>
+          <t>2026-06-24T15:28:40Z</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:52Z</t>
+          <t>2026-06-24T15:28:40Z</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:52Z</t>
+          <t>2026-06-24T15:28:40Z</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -963,11 +963,11 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>4.7e-05</v>
+        <v>0</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:52Z</t>
+          <t>2026-06-24T15:28:40Z</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Fry ORTHSC (R, live)</t>
+          <t>Fry OrthogonalizedSyntheticControl (R, live run, captured)</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:52Z</t>
+          <t>2026-06-24T15:28:41Z</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-06-24T15:03:18Z</t>
+          <t>2026-06-24T15:29:05Z</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-06-24T15:03:32Z</t>
+          <t>2026-06-24T15:29:19Z</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-06-24T15:04:04Z</t>
+          <t>2026-06-24T15:29:54Z</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-06-24T15:04:19Z</t>
+          <t>2026-06-24T15:30:10Z</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-06-24T15:04:19Z</t>
+          <t>2026-06-24T15:30:10Z</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-06-24T15:04:20Z</t>
+          <t>2026-06-24T15:30:10Z</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:23Z</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:23Z</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:43Z</t>
+          <t>2026-06-24T15:28:31Z</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R package MSCMT (vignette)</t>
+          <t>R package MSCMT (live run, captured)</t>
         </is>
       </c>
     </row>
@@ -1927,7 +1927,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Becker &amp; Klossner (2018), MSCMT vignette 'Working with package MSCMT'; pinned constants</t>
+          <t>MSCMT 1.4.4 (vignette 'Working with package MSCMT' specification); benchmarks/reference/mscmt_basque/</t>
         </is>
       </c>
     </row>
@@ -1963,10 +1963,10 @@
         <v>0.632786</v>
       </c>
       <c r="C10" t="n">
-        <v>0.63279</v>
+        <v>0.632794</v>
       </c>
       <c r="D10" t="n">
-        <v>4e-06</v>
+        <v>8e-06</v>
       </c>
     </row>
     <row r="11">
@@ -1979,10 +1979,10 @@
         <v>0.219273</v>
       </c>
       <c r="C11" t="n">
-        <v>0.21931</v>
+        <v>0.219305</v>
       </c>
       <c r="D11" t="n">
-        <v>3.7e-05</v>
+        <v>3.2e-05</v>
       </c>
     </row>
     <row r="12">
@@ -1995,10 +1995,10 @@
         <v>0.147941</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1479</v>
+        <v>0.147901</v>
       </c>
       <c r="D12" t="n">
-        <v>4.1e-05</v>
+        <v>4e-05</v>
       </c>
     </row>
     <row r="13">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:45Z</t>
+          <t>2026-06-24T15:28:34Z</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Malo et al. scm.corner (SCM-Debug)</t>
+          <t>Malo et al. scm.corner (SCM-Debug, live run, captured)</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pinned constants (benchmarks/R/scmcorner_basque.R; Malo et al. 2024, github.com/Xun90/SCM-Debug)</t>
+          <t>live captured run (benchmarks/reference/malo_basque/; Malo et al. 2024, github.com/Xun90/SCM-Debug)</t>
         </is>
       </c>
     </row>
@@ -2147,10 +2147,10 @@
         <v>0.440781</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4404</v>
+        <v>0.440444</v>
       </c>
       <c r="D10" t="n">
-        <v>0.000381</v>
+        <v>0.000337</v>
       </c>
     </row>
     <row r="11">
@@ -2163,10 +2163,10 @@
         <v>0.370264</v>
       </c>
       <c r="C11" t="n">
-        <v>0.37</v>
+        <v>0.370013</v>
       </c>
       <c r="D11" t="n">
-        <v>0.000264</v>
+        <v>0.000251</v>
       </c>
     </row>
     <row r="12">
@@ -2179,10 +2179,10 @@
         <v>0.188955</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1894</v>
+        <v>0.189436</v>
       </c>
       <c r="D12" t="n">
-        <v>0.000445</v>
+        <v>0.000481</v>
       </c>
     </row>
   </sheetData>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:48Z</t>
+          <t>2026-06-24T15:28:36Z</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:48Z</t>
+          <t>2026-06-24T15:28:37Z</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:51Z</t>
+          <t>2026-06-24T15:28:40Z</t>
         </is>
       </c>
     </row>
@@ -8515,7 +8515,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:52Z</t>
+          <t>2026-06-24T15:28:40Z</t>
         </is>
       </c>
     </row>
@@ -8843,7 +8843,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:52Z</t>
+          <t>2026-06-24T15:28:40Z</t>
         </is>
       </c>
     </row>
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:52Z</t>
+          <t>2026-06-24T15:28:40Z</t>
         </is>
       </c>
     </row>
@@ -9075,7 +9075,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fry ORTHSC (R, live)</t>
+          <t>Fry OrthogonalizedSyntheticControl (R, live run, captured)</t>
         </is>
       </c>
     </row>
@@ -9087,7 +9087,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>(R, live)</t>
+          <t>github.com/JosephPatrickFry @ 3b38684</t>
         </is>
       </c>
     </row>
@@ -9123,10 +9123,10 @@
         <v>-0.290125</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.29013</v>
+        <v>-0.290125</v>
       </c>
       <c r="D10" t="n">
-        <v>5e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -9171,10 +9171,10 @@
         <v>-0.475703</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.4757</v>
+        <v>-0.475703</v>
       </c>
       <c r="D13" t="n">
-        <v>3e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -9187,10 +9187,10 @@
         <v>-0.104547</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.1045</v>
+        <v>-0.104547</v>
       </c>
       <c r="D14" t="n">
-        <v>4.7e-05</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:00:46Z</t>
+          <t>2026-06-24T15:26:35Z</t>
         </is>
       </c>
     </row>
@@ -9667,7 +9667,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:02:52Z</t>
+          <t>2026-06-24T15:28:41Z</t>
         </is>
       </c>
     </row>
@@ -9915,7 +9915,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:03:18Z</t>
+          <t>2026-06-24T15:29:05Z</t>
         </is>
       </c>
     </row>
@@ -10275,7 +10275,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:03:32Z</t>
+          <t>2026-06-24T15:29:19Z</t>
         </is>
       </c>
     </row>
@@ -10443,7 +10443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:04:04Z</t>
+          <t>2026-06-24T15:29:54Z</t>
         </is>
       </c>
     </row>
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:04:19Z</t>
+          <t>2026-06-24T15:30:10Z</t>
         </is>
       </c>
     </row>
@@ -11019,7 +11019,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:04:19Z</t>
+          <t>2026-06-24T15:30:10Z</t>
         </is>
       </c>
     </row>
@@ -11379,7 +11379,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:04:20Z</t>
+          <t>2026-06-24T15:30:10Z</t>
         </is>
       </c>
     </row>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:05Z</t>
+          <t>2026-06-24T15:26:53Z</t>
         </is>
       </c>
     </row>
@@ -12543,7 +12543,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:08Z</t>
+          <t>2026-06-24T15:26:56Z</t>
         </is>
       </c>
     </row>
@@ -12679,7 +12679,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:29Z</t>
+          <t>2026-06-24T15:27:18Z</t>
         </is>
       </c>
     </row>
@@ -12815,7 +12815,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:22Z</t>
         </is>
       </c>
     </row>
@@ -13255,7 +13255,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:22Z</t>
         </is>
       </c>
     </row>
@@ -13471,7 +13471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:22Z</t>
         </is>
       </c>
     </row>
@@ -13751,7 +13751,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:01:33Z</t>
+          <t>2026-06-24T15:27:22Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Convert nsc_prop99 benchmark to live NSC.R reference run
Replace the hand-pinned Tian (2023) Table-2 constants with a live captured run
of the author's own NSC() (vendored at benchmarks/R/nsc_tian2023_reference.R),
executed at the selected penalty a=0.3, b=0.7 -- deterministic once the penalty
is fixed (the stochastic CV is bypassed, CI disabled). reference.R emits the
signed donor weights + effect path; the bundle is generated and the case reads
_REF_WEIGHTS/_REF_ITE and EXPECTED targets from it via load_reference/
reference_value. The live run reproduces Table 2 to the digit (every weight,
ITE 1990 -9.51 / 1995 -24.50 / 2000 -28.70); mlsynth cross-validates against it
(weight corr 0.989, no per-weight gap > 0.024).

This was the last benchmark case still on hand-pinned published constants -- the
full cross-validation corpus now runs against live or captured reference code.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/reference/comparisons.xlsx
+++ b/benchmarks/reference/comparisons.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:26:35Z</t>
+          <t>2026-06-24T15:48:17Z</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-06-24T15:26:53Z</t>
+          <t>2026-06-24T15:48:37Z</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-06-24T15:26:56Z</t>
+          <t>2026-06-24T15:48:40Z</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:18Z</t>
+          <t>2026-06-24T15:49:01Z</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:22Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:22Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:22Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:22Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -711,11 +711,11 @@
         <v>23</v>
       </c>
       <c r="C10" t="n">
-        <v>1.878871</v>
+        <v>1.877168</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:23Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Tian (2023) NSC.R (Table 2, a*=0.3, b*=0.7)</t>
+          <t>Tian (2023) NSC.R (vendored, live run, captured), a*=0.3, b*=0.7</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:23Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:31Z</t>
+          <t>2026-06-24T15:50:15Z</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:34Z</t>
+          <t>2026-06-24T15:50:17Z</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:36Z</t>
+          <t>2026-06-24T15:50:21Z</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:37Z</t>
+          <t>2026-06-24T15:50:21Z</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:40Z</t>
+          <t>2026-06-24T15:50:24Z</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:40Z</t>
+          <t>2026-06-24T15:50:24Z</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:40Z</t>
+          <t>2026-06-24T15:50:24Z</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:40Z</t>
+          <t>2026-06-24T15:50:24Z</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:41Z</t>
+          <t>2026-06-24T15:50:25Z</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-06-24T15:29:05Z</t>
+          <t>2026-06-24T15:50:50Z</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-06-24T15:29:19Z</t>
+          <t>2026-06-24T15:51:05Z</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-06-24T15:29:54Z</t>
+          <t>2026-06-24T15:51:40Z</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-06-24T15:30:10Z</t>
+          <t>2026-06-24T15:51:55Z</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-06-24T15:30:10Z</t>
+          <t>2026-06-24T15:51:55Z</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-06-24T15:30:10Z</t>
+          <t>2026-06-24T15:51:55Z</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:23Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tian (2023) NSC.R (Table 2, a*=0.3, b*=0.7)</t>
+          <t>Tian (2023) NSC.R (vendored, live run, captured), a*=0.3, b*=0.7</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NSC.R / Tian (2023) arXiv:2306.01967v1 Table 2</t>
+          <t>NSC.R / Tian (2023) arXiv:2306.01967v1 (benchmarks/reference/nsc_prop99/)</t>
         </is>
       </c>
     </row>
@@ -1627,10 +1627,10 @@
         <v>-9.054038</v>
       </c>
       <c r="C30" t="n">
-        <v>-9.5</v>
+        <v>-9.510413</v>
       </c>
       <c r="D30" t="n">
-        <v>0.445962</v>
+        <v>0.456375</v>
       </c>
     </row>
     <row r="31">
@@ -1643,10 +1643,10 @@
         <v>-22.621129</v>
       </c>
       <c r="C31" t="n">
-        <v>-24.5</v>
+        <v>-24.498297</v>
       </c>
       <c r="D31" t="n">
-        <v>1.878871</v>
+        <v>1.877168</v>
       </c>
     </row>
     <row r="32">
@@ -1659,10 +1659,10 @@
         <v>-27.011011</v>
       </c>
       <c r="C32" t="n">
-        <v>-28.7</v>
+        <v>-28.699998</v>
       </c>
       <c r="D32" t="n">
-        <v>1.688989</v>
+        <v>1.688987</v>
       </c>
     </row>
   </sheetData>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:23Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:31Z</t>
+          <t>2026-06-24T15:50:15Z</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:34Z</t>
+          <t>2026-06-24T15:50:17Z</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:36Z</t>
+          <t>2026-06-24T15:50:21Z</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:37Z</t>
+          <t>2026-06-24T15:50:21Z</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:40Z</t>
+          <t>2026-06-24T15:50:24Z</t>
         </is>
       </c>
     </row>
@@ -8515,7 +8515,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:40Z</t>
+          <t>2026-06-24T15:50:24Z</t>
         </is>
       </c>
     </row>
@@ -8843,7 +8843,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:40Z</t>
+          <t>2026-06-24T15:50:24Z</t>
         </is>
       </c>
     </row>
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:40Z</t>
+          <t>2026-06-24T15:50:24Z</t>
         </is>
       </c>
     </row>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:26:35Z</t>
+          <t>2026-06-24T15:48:17Z</t>
         </is>
       </c>
     </row>
@@ -9667,7 +9667,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:28:41Z</t>
+          <t>2026-06-24T15:50:25Z</t>
         </is>
       </c>
     </row>
@@ -9915,7 +9915,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:29:05Z</t>
+          <t>2026-06-24T15:50:50Z</t>
         </is>
       </c>
     </row>
@@ -10275,7 +10275,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:29:19Z</t>
+          <t>2026-06-24T15:51:05Z</t>
         </is>
       </c>
     </row>
@@ -10443,7 +10443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:29:54Z</t>
+          <t>2026-06-24T15:51:40Z</t>
         </is>
       </c>
     </row>
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:30:10Z</t>
+          <t>2026-06-24T15:51:55Z</t>
         </is>
       </c>
     </row>
@@ -11019,7 +11019,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:30:10Z</t>
+          <t>2026-06-24T15:51:55Z</t>
         </is>
       </c>
     </row>
@@ -11379,7 +11379,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:30:10Z</t>
+          <t>2026-06-24T15:51:55Z</t>
         </is>
       </c>
     </row>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:26:53Z</t>
+          <t>2026-06-24T15:48:37Z</t>
         </is>
       </c>
     </row>
@@ -12543,7 +12543,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:26:56Z</t>
+          <t>2026-06-24T15:48:40Z</t>
         </is>
       </c>
     </row>
@@ -12679,7 +12679,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:18Z</t>
+          <t>2026-06-24T15:49:01Z</t>
         </is>
       </c>
     </row>
@@ -12815,7 +12815,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:22Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
     </row>
@@ -13255,7 +13255,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:22Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
     </row>
@@ -13471,7 +13471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:22Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
     </row>
@@ -13751,7 +13751,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-24T15:27:22Z</t>
+          <t>2026-06-24T15:49:05Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
benchmarks: SPILLSYNTH-SAR Sudan cross-validation vs the authors' Rcpp sampler
Adds spillsynth_sudan, the empirical companion to spillsynth_sar_mc: mlsynth's
SPILLSYNTH(method=sar) on the 2011 Sudan-secession panel, cross-validated
against Sakaguchi & Tagawa's (2026) own RcppArmadillo sc_spillover run live on
the committed nonproprietary CSVs (reference.R; pinned in reference.json/.out,
manifest + provenance). Lands in the comparison workbook (comparisons.xlsx).

Compared quantities are convention-robust: rho (weakly identified -- authors'
ESS ~390 at 1e6 draws -- so a converged-posterior match, wide tol), the 2012/
2015 GDP effects, and per-country spillover shares (unit-free). All five agree:
rho 0.4357 vs 0.4315; effect_2012 -7.58 vs -7.65; effect_2015 -9.59 vs -10.0;
egypt_share 0.422 vs 0.426; kenya_share 0.144 vs 0.144.

Separate from the paper PR, per the benchmark-as-own-workstream convention.

Claude-Session: https://claude.ai/code/session_015nRd88pbMUETcrkKY1S6Hr
</commit_message>
<xml_diff>
--- a/benchmarks/reference/comparisons.xlsx
+++ b/benchmarks/reference/comparisons.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="scul_prop99" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="spillsynth_sudan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,18 +456,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>scul_prop99</t>
+          <t>spillsynth_sudan</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.13539</v>
+        <v>0.40622</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-25T16:07:00Z</t>
+          <t>2026-06-26T02:58:08Z</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -477,7 +477,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>authors' SCUL() (R, via Rscript + glmnet)</t>
+          <t>Sakaguchi-Tagawa RcppArmadillo sc_spillover (method=sar, live run on the nonproprietary panel, captured)</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,7 +503,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>scul_prop99</t>
+          <t>spillsynth_sudan</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-25T16:07:00Z</t>
+          <t>2026-06-26T02:58:08Z</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SCUL</t>
+          <t>SPILLSYNTH</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"donor_variables": ["retprice"], "outcome": "cigsale", "time": "year", "treat": "treat", "unitid": "state"}</t>
+          <t>{"mcmc_burn": 10000, "mcmc_iter": 20000, "mcmc_seed": 20251022, "method": "sar", "outcome": "GDP per capita", "p_factors": 1, "time": "year", "treat": "treated", "unitid": "country"}</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>authors' SCUL() (R, via Rscript + glmnet)</t>
+          <t>Sakaguchi-Tagawa RcppArmadillo sc_spillover (method=sar, live run on the nonproprietary panel, captured)</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>hollina/scul @ 121b588 (R, live)</t>
+          <t>Zenodo doi:10.5281/zenodo.19066186</t>
         </is>
       </c>
     </row>
@@ -604,49 +604,81 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cv lambda (median)</t>
+          <t>rho</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.02121478</v>
+        <v>0.435706</v>
       </c>
       <c r="C10" t="n">
-        <v>0.02121478</v>
+        <v>0.4315</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.004206</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ATT (post-1988 mean)</t>
+          <t>effect_2012_pct</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-13.17061</v>
+        <v>-7.579607</v>
       </c>
       <c r="C11" t="n">
-        <v>-13.306</v>
+        <v>-7.647</v>
       </c>
       <c r="D11" t="n">
-        <v>0.13539</v>
+        <v>0.06739299999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cohen's D (pre-fit)</t>
+          <t>effect_2015_pct</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.01371</v>
+        <v>-9.592779999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>0.01597</v>
+        <v>-9.999000000000001</v>
       </c>
       <c r="D12" t="n">
-        <v>0.00226</v>
+        <v>0.40622</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>egypt_spillover_share</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.421715</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.4263</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.004585</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>kenya_spillover_share</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.143824</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.1443</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.000476</v>
       </c>
     </row>
   </sheetData>

</xml_diff>